<commit_message>
Atualização automática dos dados - GitHub Actions
</commit_message>
<xml_diff>
--- a/data/Planilha_PL_CGNOR.xlsx
+++ b/data/Planilha_PL_CGNOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.chaves\Documents\SEGES\Projetos\Monitoramento_Parlamentar_DELOG\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\Documents\SEGES\Projetos\Monitoramento_Parlamentar_CGNOR_DELOG\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C31D290-C4B5-4B0F-9A38-9B1C47ABDF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86642324-7B4F-400B-BBE1-B5614DAC8C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DADOS PLs" sheetId="1" r:id="rId1"/>
@@ -2900,34 +2900,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BI156"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="48.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="31.42578125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="23.140625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" style="7" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" style="7" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" style="7" customWidth="1"/>
-    <col min="10" max="10" width="20.5703125" style="7" customWidth="1"/>
-    <col min="11" max="11" width="22.42578125" style="7" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="7" customWidth="1"/>
-    <col min="13" max="13" width="17.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.5703125" style="7" customWidth="1"/>
-    <col min="15" max="17" width="17.42578125" style="7" customWidth="1"/>
-    <col min="18" max="18" width="31.140625" style="7" customWidth="1"/>
-    <col min="19" max="19" width="20.28515625" style="7" customWidth="1"/>
-    <col min="20" max="20" width="26.7109375" style="7" customWidth="1"/>
-    <col min="21" max="21" width="31.42578125" style="7" customWidth="1"/>
+    <col min="1" max="1" width="3.3828125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.3828125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="48.84375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="31.3828125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="23.15234375" style="7" customWidth="1"/>
+    <col min="7" max="7" width="25.3046875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="16.69140625" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.3046875" style="7" customWidth="1"/>
+    <col min="10" max="10" width="20.53515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="22.3828125" style="7" customWidth="1"/>
+    <col min="12" max="12" width="13.84375" style="7" customWidth="1"/>
+    <col min="13" max="13" width="17.3828125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.53515625" style="7" customWidth="1"/>
+    <col min="15" max="17" width="17.3828125" style="7" customWidth="1"/>
+    <col min="18" max="18" width="31.15234375" style="7" customWidth="1"/>
+    <col min="19" max="19" width="20.3046875" style="7" customWidth="1"/>
+    <col min="20" max="20" width="26.69140625" style="7" customWidth="1"/>
+    <col min="21" max="21" width="31.3828125" style="7" customWidth="1"/>
     <col min="22" max="22" width="18" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="44.7109375" style="14" customWidth="1"/>
-    <col min="24" max="24" width="57.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.140625" style="6" customWidth="1"/>
+    <col min="23" max="23" width="44.69140625" style="14" customWidth="1"/>
+    <col min="24" max="24" width="57.69140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.15234375" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:61" x14ac:dyDescent="0.4">
       <c r="A1" s="59" t="s">
         <v>0</v>
       </c>
@@ -2956,7 +2956,7 @@
       <c r="X1" s="60"/>
       <c r="Y1" s="46"/>
     </row>
-    <row r="2" spans="1:61" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:61" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:61" s="6" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:61" s="6" customFormat="1" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3146,7 +3146,7 @@
       <c r="BH3"/>
       <c r="BI3" s="13"/>
     </row>
-    <row r="4" spans="1:61" ht="225" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:61" ht="204" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:61" ht="252" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:61" ht="237.9" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:61" ht="150" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:61" ht="131.15" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:61" ht="120" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:61" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3448,7 +3448,7 @@
       <c r="X7" s="52"/>
       <c r="Y7" s="3"/>
     </row>
-    <row r="8" spans="1:61" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:61" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3525,7 +3525,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:61" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:61" ht="72.900000000000006" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:61" ht="345" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:61" ht="306" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:61" ht="315" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:61" ht="276.89999999999998" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:61" ht="90" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:61" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:61" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:61" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3910,7 +3910,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:61" ht="195" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:61" ht="174.9" x14ac:dyDescent="0.4">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:61" ht="225" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:61" ht="204" x14ac:dyDescent="0.4">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:61" ht="255" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:61" ht="233.15" x14ac:dyDescent="0.4">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -4141,7 +4141,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" ht="189.45" x14ac:dyDescent="0.4">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -4216,7 +4216,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="210" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="204" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -4293,7 +4293,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" ht="160.30000000000001" x14ac:dyDescent="0.4">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="160.30000000000001" x14ac:dyDescent="0.4">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="255" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" ht="233.15" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -4524,7 +4524,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="150" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -4601,7 +4601,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="285" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" ht="247.75" x14ac:dyDescent="0.4">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="26" spans="1:25" ht="180" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -4986,7 +4986,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="28" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" ht="160.30000000000001" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="29" spans="1:25" ht="180" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="160.30000000000001" x14ac:dyDescent="0.4">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -5140,7 +5140,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" ht="189.45" x14ac:dyDescent="0.4">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -5215,7 +5215,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="102" x14ac:dyDescent="0.4">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -5292,7 +5292,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="32" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="33" spans="1:25" ht="240" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" ht="204" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -5440,7 +5440,7 @@
       <c r="X33" s="3"/>
       <c r="Y33" s="3"/>
     </row>
-    <row r="34" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -5513,7 +5513,7 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
-    <row r="35" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -5586,7 +5586,7 @@
       <c r="X35" s="3"/>
       <c r="Y35" s="3"/>
     </row>
-    <row r="36" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -5659,7 +5659,7 @@
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
     </row>
-    <row r="37" spans="1:25" ht="240" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" ht="204" x14ac:dyDescent="0.4">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -5732,7 +5732,7 @@
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
     </row>
-    <row r="38" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -5805,7 +5805,7 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
     </row>
-    <row r="39" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" ht="102" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -5878,7 +5878,7 @@
       <c r="X39" s="3"/>
       <c r="Y39" s="3"/>
     </row>
-    <row r="40" spans="1:25" ht="220.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" ht="190.3" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -5951,7 +5951,7 @@
       <c r="X40" s="3"/>
       <c r="Y40" s="3"/>
     </row>
-    <row r="41" spans="1:25" ht="240" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="218.6" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -6024,7 +6024,7 @@
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
     </row>
-    <row r="42" spans="1:25" ht="240" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" ht="204" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -6097,7 +6097,7 @@
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
     </row>
-    <row r="43" spans="1:25" ht="300" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" ht="247.75" x14ac:dyDescent="0.4">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -6170,7 +6170,7 @@
       <c r="X43" s="3"/>
       <c r="Y43" s="3"/>
     </row>
-    <row r="44" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" ht="204" x14ac:dyDescent="0.4">
       <c r="A44" s="2">
         <v>42</v>
       </c>
@@ -6243,7 +6243,7 @@
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
     </row>
-    <row r="45" spans="1:25" ht="165" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" ht="145.75" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
         <v>43</v>
       </c>
@@ -6316,7 +6316,7 @@
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
     </row>
-    <row r="46" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -6389,7 +6389,7 @@
       <c r="X46" s="3"/>
       <c r="Y46" s="3"/>
     </row>
-    <row r="47" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" ht="174.9" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -6462,7 +6462,7 @@
       <c r="X47" s="3"/>
       <c r="Y47" s="3"/>
     </row>
-    <row r="48" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -6535,7 +6535,7 @@
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
     </row>
-    <row r="49" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:25" ht="102" x14ac:dyDescent="0.4">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -6608,7 +6608,7 @@
       <c r="X49" s="3"/>
       <c r="Y49" s="3"/>
     </row>
-    <row r="50" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:25" ht="174.9" x14ac:dyDescent="0.4">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -6681,7 +6681,7 @@
       <c r="X50" s="3"/>
       <c r="Y50" s="3"/>
     </row>
-    <row r="51" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:25" ht="72.900000000000006" x14ac:dyDescent="0.4">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -6754,7 +6754,7 @@
       <c r="X51" s="3"/>
       <c r="Y51" s="3"/>
     </row>
-    <row r="52" spans="1:25" ht="150" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:25" ht="131.15" x14ac:dyDescent="0.4">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -6827,7 +6827,7 @@
       <c r="X52" s="3"/>
       <c r="Y52" s="3"/>
     </row>
-    <row r="53" spans="1:25" ht="195" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" ht="174.9" x14ac:dyDescent="0.4">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -6900,7 +6900,7 @@
       <c r="X53" s="3"/>
       <c r="Y53" s="3"/>
     </row>
-    <row r="54" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:25" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -6973,7 +6973,7 @@
       <c r="X54" s="3"/>
       <c r="Y54" s="3"/>
     </row>
-    <row r="55" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -7046,7 +7046,7 @@
       <c r="X55" s="3"/>
       <c r="Y55" s="3"/>
     </row>
-    <row r="56" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A56" s="2">
         <v>54</v>
       </c>
@@ -7119,7 +7119,7 @@
       <c r="X56" s="3"/>
       <c r="Y56" s="3"/>
     </row>
-    <row r="57" spans="1:25" ht="255" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" ht="218.6" x14ac:dyDescent="0.4">
       <c r="A57" s="2">
         <v>55</v>
       </c>
@@ -7192,7 +7192,7 @@
       <c r="X57" s="3"/>
       <c r="Y57" s="3"/>
     </row>
-    <row r="58" spans="1:25" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -7265,7 +7265,7 @@
       <c r="X58" s="3"/>
       <c r="Y58" s="3"/>
     </row>
-    <row r="59" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A59" s="2">
         <v>57</v>
       </c>
@@ -7338,7 +7338,7 @@
       <c r="X59" s="3"/>
       <c r="Y59" s="3"/>
     </row>
-    <row r="60" spans="1:25" ht="150" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" ht="131.15" x14ac:dyDescent="0.4">
       <c r="A60" s="2">
         <v>58</v>
       </c>
@@ -7411,7 +7411,7 @@
       <c r="X60" s="3"/>
       <c r="Y60" s="3"/>
     </row>
-    <row r="61" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" ht="189.45" x14ac:dyDescent="0.4">
       <c r="A61" s="2">
         <v>59</v>
       </c>
@@ -7484,7 +7484,7 @@
       <c r="X61" s="3"/>
       <c r="Y61" s="3"/>
     </row>
-    <row r="62" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" ht="72.900000000000006" x14ac:dyDescent="0.4">
       <c r="A62" s="3">
         <v>60</v>
       </c>
@@ -7557,7 +7557,7 @@
       <c r="X62" s="3"/>
       <c r="Y62" s="3"/>
     </row>
-    <row r="63" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A63" s="3">
         <v>61</v>
       </c>
@@ -7624,7 +7624,7 @@
       <c r="X63" s="3"/>
       <c r="Y63" s="3"/>
     </row>
-    <row r="64" spans="1:25" ht="345" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" ht="306" x14ac:dyDescent="0.4">
       <c r="A64" s="3">
         <v>62</v>
       </c>
@@ -7697,7 +7697,7 @@
       <c r="X64" s="3"/>
       <c r="Y64" s="3"/>
     </row>
-    <row r="65" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" ht="102" x14ac:dyDescent="0.4">
       <c r="A65" s="3">
         <v>63</v>
       </c>
@@ -7770,7 +7770,7 @@
       <c r="X65" s="3"/>
       <c r="Y65" s="3"/>
     </row>
-    <row r="66" spans="1:25" ht="105" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A66" s="3">
         <v>64</v>
       </c>
@@ -7843,7 +7843,7 @@
       <c r="X66" s="3"/>
       <c r="Y66" s="3"/>
     </row>
-    <row r="67" spans="1:25" ht="225" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" ht="218.6" x14ac:dyDescent="0.4">
       <c r="A67" s="3">
         <v>65</v>
       </c>
@@ -7910,7 +7910,7 @@
       <c r="X67" s="3"/>
       <c r="Y67" s="3"/>
     </row>
-    <row r="68" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" ht="87.45" x14ac:dyDescent="0.4">
       <c r="A68" s="3">
         <v>66</v>
       </c>
@@ -7983,7 +7983,7 @@
       <c r="X68" s="3"/>
       <c r="Y68" s="3"/>
     </row>
-    <row r="69" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" ht="116.6" x14ac:dyDescent="0.4">
       <c r="A69" s="3">
         <v>67</v>
       </c>
@@ -8056,7 +8056,7 @@
       <c r="X69" s="3"/>
       <c r="Y69" s="3"/>
     </row>
-    <row r="70" spans="1:25" ht="150" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:25" ht="131.15" x14ac:dyDescent="0.4">
       <c r="A70" s="3">
         <v>68</v>
       </c>
@@ -8127,432 +8127,432 @@
       <c r="X70" s="3"/>
       <c r="Y70" s="3"/>
     </row>
-    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W71" s="8"/>
       <c r="X71"/>
       <c r="Y71"/>
     </row>
-    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W72" s="8"/>
       <c r="X72"/>
       <c r="Y72"/>
     </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W73" s="8"/>
       <c r="X73"/>
       <c r="Y73"/>
     </row>
-    <row r="74" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W74" s="8"/>
       <c r="X74"/>
       <c r="Y74"/>
     </row>
-    <row r="75" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W75" s="8"/>
       <c r="X75"/>
       <c r="Y75"/>
     </row>
-    <row r="76" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W76" s="8"/>
       <c r="X76"/>
       <c r="Y76"/>
     </row>
-    <row r="77" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W77" s="8"/>
       <c r="X77"/>
       <c r="Y77"/>
     </row>
-    <row r="78" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W78" s="8"/>
       <c r="X78"/>
       <c r="Y78"/>
     </row>
-    <row r="79" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W79" s="8"/>
       <c r="X79"/>
       <c r="Y79"/>
     </row>
-    <row r="80" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" x14ac:dyDescent="0.4">
       <c r="W80" s="8"/>
       <c r="X80"/>
       <c r="Y80"/>
     </row>
-    <row r="81" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="81" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W81" s="8"/>
       <c r="X81"/>
       <c r="Y81"/>
     </row>
-    <row r="82" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="82" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W82" s="8"/>
       <c r="X82"/>
       <c r="Y82"/>
     </row>
-    <row r="83" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="83" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W83" s="8"/>
       <c r="X83"/>
       <c r="Y83"/>
     </row>
-    <row r="84" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="84" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W84" s="8"/>
       <c r="X84"/>
       <c r="Y84"/>
     </row>
-    <row r="85" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="85" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W85" s="8"/>
       <c r="X85"/>
       <c r="Y85"/>
     </row>
-    <row r="86" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="86" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W86" s="8"/>
       <c r="X86"/>
       <c r="Y86"/>
     </row>
-    <row r="87" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="87" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W87" s="8"/>
       <c r="X87"/>
       <c r="Y87"/>
     </row>
-    <row r="88" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="88" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W88" s="8"/>
       <c r="X88"/>
       <c r="Y88"/>
     </row>
-    <row r="89" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="89" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W89" s="8"/>
       <c r="X89"/>
       <c r="Y89"/>
     </row>
-    <row r="90" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="90" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W90" s="8"/>
       <c r="X90"/>
       <c r="Y90"/>
     </row>
-    <row r="91" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="91" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W91" s="8"/>
       <c r="X91"/>
       <c r="Y91"/>
     </row>
-    <row r="92" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="92" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W92" s="8"/>
       <c r="X92"/>
       <c r="Y92"/>
     </row>
-    <row r="93" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="93" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W93" s="8"/>
       <c r="X93"/>
       <c r="Y93"/>
     </row>
-    <row r="94" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="94" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W94" s="8"/>
       <c r="X94"/>
       <c r="Y94"/>
     </row>
-    <row r="95" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="95" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W95" s="8"/>
       <c r="X95"/>
       <c r="Y95"/>
     </row>
-    <row r="96" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="96" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W96" s="8"/>
       <c r="X96"/>
       <c r="Y96"/>
     </row>
-    <row r="97" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="97" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W97" s="8"/>
       <c r="X97"/>
       <c r="Y97"/>
     </row>
-    <row r="98" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="98" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W98" s="8"/>
       <c r="X98"/>
       <c r="Y98"/>
     </row>
-    <row r="99" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="99" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W99" s="8"/>
       <c r="X99"/>
       <c r="Y99"/>
     </row>
-    <row r="100" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="100" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W100" s="8"/>
       <c r="X100"/>
       <c r="Y100"/>
     </row>
-    <row r="101" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="101" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W101" s="8"/>
       <c r="X101"/>
       <c r="Y101"/>
     </row>
-    <row r="102" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="102" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W102" s="8"/>
       <c r="X102"/>
       <c r="Y102"/>
     </row>
-    <row r="103" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="103" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W103" s="8"/>
       <c r="X103"/>
       <c r="Y103"/>
     </row>
-    <row r="104" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="104" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W104" s="8"/>
       <c r="X104"/>
       <c r="Y104"/>
     </row>
-    <row r="105" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="105" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W105" s="8"/>
       <c r="X105"/>
       <c r="Y105"/>
     </row>
-    <row r="106" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="106" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W106" s="8"/>
       <c r="X106"/>
       <c r="Y106"/>
     </row>
-    <row r="107" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="107" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W107" s="8"/>
       <c r="X107"/>
       <c r="Y107"/>
     </row>
-    <row r="108" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="108" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W108" s="8"/>
       <c r="X108"/>
       <c r="Y108"/>
     </row>
-    <row r="109" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="109" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W109" s="8"/>
       <c r="X109"/>
       <c r="Y109"/>
     </row>
-    <row r="110" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="110" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W110" s="8"/>
       <c r="X110"/>
       <c r="Y110"/>
     </row>
-    <row r="111" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="111" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W111" s="8"/>
       <c r="X111"/>
       <c r="Y111"/>
     </row>
-    <row r="112" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="112" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W112" s="8"/>
       <c r="X112"/>
       <c r="Y112"/>
     </row>
-    <row r="113" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="113" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W113" s="8"/>
       <c r="X113"/>
       <c r="Y113"/>
     </row>
-    <row r="114" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="114" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W114" s="8"/>
       <c r="X114"/>
       <c r="Y114"/>
     </row>
-    <row r="115" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="115" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W115" s="8"/>
       <c r="X115"/>
       <c r="Y115"/>
     </row>
-    <row r="116" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="116" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W116" s="8"/>
       <c r="X116"/>
       <c r="Y116"/>
     </row>
-    <row r="117" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="117" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W117" s="8"/>
       <c r="X117"/>
       <c r="Y117"/>
     </row>
-    <row r="118" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="118" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W118" s="8"/>
       <c r="X118"/>
       <c r="Y118"/>
     </row>
-    <row r="119" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="119" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W119" s="8"/>
       <c r="X119"/>
       <c r="Y119"/>
     </row>
-    <row r="120" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="120" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W120" s="8"/>
       <c r="X120"/>
       <c r="Y120"/>
     </row>
-    <row r="121" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="121" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W121" s="8"/>
       <c r="X121"/>
       <c r="Y121"/>
     </row>
-    <row r="122" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="122" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W122" s="8"/>
       <c r="X122"/>
       <c r="Y122"/>
     </row>
-    <row r="123" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="123" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W123" s="8"/>
       <c r="X123"/>
       <c r="Y123"/>
     </row>
-    <row r="124" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="124" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W124" s="8"/>
       <c r="X124"/>
       <c r="Y124"/>
     </row>
-    <row r="125" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="125" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W125" s="8"/>
       <c r="X125"/>
       <c r="Y125"/>
     </row>
-    <row r="126" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="126" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W126" s="8"/>
       <c r="X126"/>
       <c r="Y126"/>
     </row>
-    <row r="127" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="127" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W127" s="8"/>
       <c r="X127"/>
       <c r="Y127"/>
     </row>
-    <row r="128" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="128" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W128" s="8"/>
       <c r="X128"/>
       <c r="Y128"/>
     </row>
-    <row r="129" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="129" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W129" s="8"/>
       <c r="X129"/>
       <c r="Y129"/>
     </row>
-    <row r="130" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="130" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W130" s="8"/>
       <c r="X130"/>
       <c r="Y130"/>
     </row>
-    <row r="131" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="131" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W131" s="8"/>
       <c r="X131"/>
       <c r="Y131"/>
     </row>
-    <row r="132" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="132" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W132" s="8"/>
       <c r="X132"/>
       <c r="Y132"/>
     </row>
-    <row r="133" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="133" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W133" s="8"/>
       <c r="X133"/>
       <c r="Y133"/>
     </row>
-    <row r="134" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="134" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W134" s="8"/>
       <c r="X134"/>
       <c r="Y134"/>
     </row>
-    <row r="135" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="135" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W135" s="8"/>
       <c r="X135"/>
       <c r="Y135"/>
     </row>
-    <row r="136" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="136" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W136" s="8"/>
       <c r="X136"/>
       <c r="Y136"/>
     </row>
-    <row r="137" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="137" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W137" s="8"/>
       <c r="X137"/>
       <c r="Y137"/>
     </row>
-    <row r="138" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="138" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W138" s="8"/>
       <c r="X138"/>
       <c r="Y138"/>
     </row>
-    <row r="139" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="139" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W139" s="8"/>
       <c r="X139"/>
       <c r="Y139"/>
     </row>
-    <row r="140" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="140" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W140" s="8"/>
       <c r="X140"/>
       <c r="Y140"/>
     </row>
-    <row r="141" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="141" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W141" s="8"/>
       <c r="X141"/>
       <c r="Y141"/>
     </row>
-    <row r="142" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="142" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W142" s="8"/>
       <c r="X142"/>
       <c r="Y142"/>
     </row>
-    <row r="143" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="143" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W143" s="8"/>
       <c r="X143"/>
       <c r="Y143"/>
     </row>
-    <row r="144" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="144" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W144" s="8"/>
       <c r="X144"/>
       <c r="Y144"/>
     </row>
-    <row r="145" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="145" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W145" s="8"/>
       <c r="X145"/>
       <c r="Y145"/>
     </row>
-    <row r="146" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="146" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W146" s="8"/>
       <c r="X146"/>
       <c r="Y146"/>
     </row>
-    <row r="147" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="147" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W147" s="8"/>
       <c r="X147"/>
       <c r="Y147"/>
     </row>
-    <row r="148" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="148" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W148" s="8"/>
       <c r="X148"/>
       <c r="Y148"/>
     </row>
-    <row r="149" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="149" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W149" s="8"/>
       <c r="X149"/>
       <c r="Y149"/>
     </row>
-    <row r="150" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="150" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W150" s="8"/>
       <c r="X150"/>
       <c r="Y150"/>
     </row>
-    <row r="151" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="151" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W151" s="8"/>
       <c r="X151"/>
       <c r="Y151"/>
     </row>
-    <row r="152" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="152" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W152" s="8"/>
       <c r="X152"/>
       <c r="Y152"/>
     </row>
-    <row r="153" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="153" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W153" s="8"/>
       <c r="X153"/>
       <c r="Y153"/>
     </row>
-    <row r="154" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="154" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W154" s="8"/>
       <c r="X154"/>
       <c r="Y154"/>
     </row>
-    <row r="155" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="155" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W155" s="8"/>
       <c r="X155"/>
       <c r="Y155"/>
     </row>
-    <row r="156" spans="23:25" x14ac:dyDescent="0.25">
+    <row r="156" spans="23:25" x14ac:dyDescent="0.4">
       <c r="W156" s="25"/>
       <c r="X156" s="19"/>
       <c r="Y156" s="19"/>
@@ -8600,13 +8600,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C047E11-A66A-4292-8601-E7F8F1BFF37E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a" xsi:nil="true"/>
+    <SharedWithUsers xmlns="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a">
+      <UserInfo>
+        <DisplayName>Manuela Deolinda dos Santos da Silva Pires</DisplayName>
+        <AccountId>20</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Marina do Be Nascentes Marcondes de França Ferreira</DisplayName>
+        <AccountId>22</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Adriano Dutra Carrijo</DisplayName>
+        <AccountId>245</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100D1C650F3C26BBF44B7C6A67686292D0C" ma:contentTypeVersion="18" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="5c1dbdf1a86738ed3f1a12087e38d711">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e" xmlns:ns3="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00e0d89b555613befc0171f33fb080da" ns2:_="" ns3:_="">
     <xsd:import namespace="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e"/>
@@ -8855,44 +8892,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24A46A21-98CA-4F3F-9A10-B3D60D1AE307}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a" xsi:nil="true"/>
-    <SharedWithUsers xmlns="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a">
-      <UserInfo>
-        <DisplayName>Manuela Deolinda dos Santos da Silva Pires</DisplayName>
-        <AccountId>20</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Marina do Be Nascentes Marcondes de França Ferreira</DisplayName>
-        <AccountId>22</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Adriano Dutra Carrijo</DisplayName>
-        <AccountId>245</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B67EE7A-E355-43DD-A56B-FB5A70ADFC8C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e"/>
+    <ds:schemaRef ds:uri="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC21D672-53B8-4449-B3DC-79DE8A0509DC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8909,23 +8928,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24A46A21-98CA-4F3F-9A10-B3D60D1AE307}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B67EE7A-E355-43DD-A56B-FB5A70ADFC8C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cd7d596d-832d-45e0-89a4-fa9e3b7aa31e"/>
-    <ds:schemaRef ds:uri="ea0f54e9-5601-4107-94f4-6fbe9e4cb98a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>